<commit_message>
add browser compatibility row to the comparison table
</commit_message>
<xml_diff>
--- a/comparison-all-wind-layer-package.xlsx
+++ b/comparison-all-wind-layer-package.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zifanwang/Documents/GitHub/mapbox-exif-layer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7BFC23A-0A39-8C44-AD68-DA15C5A5D9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6A8FC2A-BDB4-F545-9EDD-BD959F4DB1C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4840" yWindow="7240" windowWidth="28040" windowHeight="17440" xr2:uid="{D8B2BD75-BB0B-2440-9919-EF3F6004A2DF}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="27000" xr2:uid="{D8B2BD75-BB0B-2440-9919-EF3F6004A2DF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="comparison-all-wind-layer-packa" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>mapbox-exif-layer</t>
   </si>
@@ -108,13 +108,25 @@
   </si>
   <si>
     <t>Yes (only possible for maplibre but not mapbox)</t>
+  </si>
+  <si>
+    <t>Browser on mobile device support</t>
+  </si>
+  <si>
+    <t>No (very likely to lose WebGL context)</t>
+  </si>
+  <si>
+    <t>Yes (native)</t>
+  </si>
+  <si>
+    <t>Yes (depends on deck.gl)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -123,8 +135,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="12"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
@@ -171,18 +189,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -519,15 +540,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{448EF52C-0849-B645-B17D-38063DCAEFB7}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="24.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="26.83203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="46" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -539,7 +559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -553,7 +573,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="69" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -567,7 +587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="69" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
@@ -581,7 +601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="46" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -595,7 +615,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="69" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -609,7 +629,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -623,17 +643,31 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="69" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="115" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>